<commit_message>
Added new RDF data schemes and visual schemes for environment-table02-03, and fixed XLSX spreadsheet for environment-table03
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table03.xlsx
+++ b/sources/table_normalization/xlsx/environment-table03.xlsx
@@ -97,7 +97,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -227,24 +227,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -257,7 +242,22 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -540,19 +540,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="33" customHeight="1">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="11" t="s">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="12"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1">
@@ -564,7 +564,7 @@
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="19" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1">
@@ -578,7 +578,7 @@
       <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1">
@@ -594,7 +594,7 @@
       <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="19" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1">
@@ -612,7 +612,7 @@
       <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="19" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1">
@@ -633,19 +633,19 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="20"/>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="14" t="s">
         <v>5</v>
       </c>
     </row>
@@ -662,19 +662,19 @@
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="33" customHeight="1">
-      <c r="A10" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="14" t="s">
+      <c r="A10" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="19" t="s">
         <v>2</v>
       </c>
       <c r="B11" s="6">
@@ -686,7 +686,7 @@
       <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="19" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="6">
@@ -700,7 +700,7 @@
       <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="19" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="6">
@@ -716,7 +716,7 @@
       <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="19" t="s">
         <v>5</v>
       </c>
       <c r="B14" s="6">
@@ -734,7 +734,7 @@
       <c r="F14" s="7"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="19" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="6">
@@ -755,19 +755,19 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="20"/>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="14" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>